<commit_message>
Added GongGetUUID new gong
</commit_message>
<xml_diff>
--- a/test/test/go/tests/serialize_test.xlsx
+++ b/test/test/go/tests/serialize_test.xlsx
@@ -12,16 +12,16 @@
     <sheet name="AstructBstructUse" sheetId="4" r:id="rId7"/>
     <sheet name="Bstruct" sheetId="5" r:id="rId8"/>
     <sheet name="Dstruct" sheetId="6" r:id="rId9"/>
-    <sheet name="Fstruct" sheetId="7" r:id="rId10"/>
+    <sheet name="F012345678901234567890123456789" sheetId="7" r:id="rId10"/>
     <sheet name="Gstruct" sheetId="8" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'Astruct'!$A$1:$AK$1</definedName>
+    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'Astruct'!$A$1:$AF$1</definedName>
     <definedName hidden="true" localSheetId="1" name="_xlnm._FilterDatabase">'AstructBstruct2Use'!$A$1:$B$1</definedName>
     <definedName hidden="true" localSheetId="2" name="_xlnm._FilterDatabase">'AstructBstructUse'!$A$1:$B$1</definedName>
     <definedName hidden="true" localSheetId="3" name="_xlnm._FilterDatabase">'Bstruct'!$A$1:$D$1</definedName>
     <definedName hidden="true" localSheetId="4" name="_xlnm._FilterDatabase">'Dstruct'!$A$1:$D$1</definedName>
-    <definedName hidden="true" localSheetId="5" name="_xlnm._FilterDatabase">'Fstruct'!$A$1:$B$1</definedName>
+    <definedName hidden="true" localSheetId="5" name="_xlnm._FilterDatabase">'F012345678901234567890123456789'!$A$1:$B$1</definedName>
     <definedName hidden="true" localSheetId="6" name="_xlnm._FilterDatabase">'Gstruct'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
@@ -29,11 +29,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>Name</t>
   </si>
   <si>
+    <t>Field</t>
+  </si>
+  <si>
     <t>Associationtob</t>
   </si>
   <si>
@@ -118,24 +121,6 @@
     <t>AnAstruct</t>
   </si>
   <si>
-    <t>StructRef</t>
-  </si>
-  <si>
-    <t>FieldRef</t>
-  </si>
-  <si>
-    <t>EnumIntRef</t>
-  </si>
-  <si>
-    <t>EnumStringRef</t>
-  </si>
-  <si>
-    <t>EnumValue</t>
-  </si>
-  <si>
-    <t>ConstIdentifierValue</t>
-  </si>
-  <si>
     <t>TextFieldBespokeSize</t>
   </si>
   <si>
@@ -143,6 +128,9 @@
   </si>
   <si>
     <t>A1</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>B1</t>
@@ -150,9 +138,6 @@
   <si>
     <t>B2
 B1</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>0001-01-01 00:00:00 +0000 UTC</t>
@@ -215,17 +200,15 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
+      <family val="2"/>
       <b val="1"/>
-      <sz val="11"/>
       <color/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -526,39 +509,7 @@
   <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="1" width="6"/>
-    <col customWidth="true" max="2" min="2" style="1" width="16"/>
-    <col customWidth="true" max="3" min="3" style="1" width="12"/>
-    <col customWidth="true" max="4" min="4" style="1" width="25"/>
-    <col customWidth="true" max="5" min="5" style="1" width="31"/>
-    <col customWidth="true" max="6" min="6" style="1" width="12"/>
-    <col customWidth="true" max="7" min="7" style="1" width="14"/>
-    <col customWidth="true" max="8" min="8" style="1" width="7"/>
-    <col customWidth="true" max="9" min="9" style="1" width="9"/>
-    <col customWidth="true" max="10" min="10" style="1" width="7"/>
-    <col customWidth="true" max="11" min="11" style="1" width="12"/>
-    <col customWidth="true" max="12" min="12" style="1" width="7"/>
-    <col customWidth="true" max="13" min="13" style="1" width="13"/>
-    <col customWidth="true" max="14" min="14" style="1" width="9"/>
-    <col customWidth="true" max="15" min="15" style="1" width="10"/>
-    <col customWidth="true" max="16" min="16" style="1" width="9"/>
-    <col customWidth="true" max="19" min="17" style="1" width="10"/>
-    <col customWidth="true" max="20" min="20" style="1" width="11"/>
-    <col customWidth="true" max="21" min="21" style="1" width="12"/>
-    <col customWidth="true" max="22" min="22" style="1" width="10"/>
-    <col customWidth="true" max="23" min="23" style="1" width="21"/>
-    <col customWidth="true" max="24" min="24" style="1" width="11"/>
-    <col customWidth="true" max="25" min="25" style="1" width="12"/>
-    <col customWidth="true" max="26" min="26" style="1" width="17"/>
-    <col customWidth="true" max="27" min="27" style="1" width="15"/>
-    <col customWidth="true" max="28" min="28" style="1" width="16"/>
-    <col customWidth="true" max="30" min="29" style="1" width="11"/>
-    <col customWidth="true" max="31" min="31" style="1" width="10"/>
-    <col customWidth="true" max="32" min="32" style="1" width="12"/>
-    <col customWidth="true" max="33" min="33" style="1" width="15"/>
-    <col customWidth="true" max="34" min="34" style="1" width="11"/>
-    <col customWidth="true" max="36" min="35" style="1" width="22"/>
-    <col customWidth="true" max="37" min="37" style="1" width="10"/>
+    <col max="32" min="1" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -658,363 +609,303 @@
       <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AH1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AI1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AJ1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AK1" s="2" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="I2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>40</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="P2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="S2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="X2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="Z2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AB2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AC2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AD2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AF2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AG2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AH2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AI2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AJ2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AK2" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="I3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>40</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="W3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="X3" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="Z3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AB3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AC3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AD3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AF3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AG3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AH3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AI3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AJ3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AK3" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="I4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>40</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="R4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="V4" s="1" t="s">
         <v>47</v>
       </c>
       <c r="W4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="X4" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="Z4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AB4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AC4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AD4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AG4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AH4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AI4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AJ4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AK4" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$AK$1"/>
+  <autoFilter ref="$A$1:$AF$1"/>
 </worksheet>
 </file>
 
@@ -1023,8 +914,7 @@
   <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="1" width="6"/>
-    <col customWidth="true" max="2" min="2" style="1" width="10"/>
+    <col max="2" min="1" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1032,7 +922,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1045,8 +935,7 @@
   <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="1" width="6"/>
-    <col customWidth="true" max="2" min="2" style="1" width="10"/>
+    <col max="2" min="1" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1054,7 +943,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1067,10 +956,7 @@
   <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="1" width="6"/>
-    <col customWidth="true" max="2" min="2" style="1" width="12"/>
-    <col customWidth="true" max="3" min="3" style="1" width="13"/>
-    <col customWidth="true" max="4" min="4" style="1" width="10"/>
+    <col max="4" min="1" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1078,41 +964,41 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1125,10 +1011,7 @@
   <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="1" width="6"/>
-    <col customWidth="true" max="2" min="2" style="1" width="12"/>
-    <col customWidth="true" max="3" min="3" style="1" width="9"/>
-    <col customWidth="true" max="4" min="4" style="1" width="10"/>
+    <col max="4" min="1" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1136,13 +1019,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1155,7 +1038,7 @@
   <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="2" min="1" style="1" width="6"/>
+    <col max="2" min="1" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1163,7 +1046,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1176,10 +1059,7 @@
   <sheetPr filterMode="true"/>
   <dimension ref="A1"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="1" width="6"/>
-    <col customWidth="true" max="2" min="2" style="1" width="12"/>
-    <col customWidth="true" max="3" min="3" style="1" width="13"/>
-    <col customWidth="true" max="4" min="4" style="1" width="10"/>
+    <col max="4" min="1" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1187,13 +1067,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>